<commit_message>
[1216] [Backend]-Add sys_event_log column in report table, a new API /reports/script for no_auth using and a new upload_report.py file for testing.
</commit_message>
<xml_diff>
--- a/backend/app/test_data/PTL_Workshop/test_report_20251015_135924.xlsx
+++ b/backend/app/test_data/PTL_Workshop/test_report_20251015_135924.xlsx
@@ -1,21 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erniewux\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D78E4D-F76C-4D2C-B8BE-4AE9FDE6399A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="28800" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="BT Test Report" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -142,7 +149,7 @@
     <t>op_name</t>
   </si>
   <si>
-    <t>Leo</t>
+    <t>Admin</t>
   </si>
   <si>
     <t>date</t>
@@ -418,35 +425,373 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-&quot;NT$&quot;* #,##0.00_-;\-&quot;NT$&quot;* #,##0.00_-;_-&quot;NT$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-&quot;NT$&quot;* #,##0_-;\-&quot;NT$&quot;* #,##0_-;_-&quot;NT$&quot;* &quot;-&quot;_-;_-@_-"/>
+  </numFmts>
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -454,29 +799,314 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -761,32 +1391,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D94"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="21" spans="1:1">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-    </row>
-    <row r="3" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    </row>
+    <row r="3" ht="18.75" spans="1:1">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -794,7 +1421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -802,7 +1429,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -810,17 +1437,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+    <row r="9" ht="18.75" spans="1:1">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -828,7 +1455,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -836,7 +1463,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -844,7 +1471,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -852,7 +1479,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -860,7 +1487,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -868,7 +1495,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -876,7 +1503,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -884,7 +1511,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -892,7 +1519,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -900,7 +1527,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -908,7 +1535,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -916,7 +1543,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -924,7 +1551,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -932,7 +1559,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -940,7 +1567,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -948,7 +1575,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -956,12 +1583,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
+    <row r="28" ht="18.75" spans="1:1">
+      <c r="A28" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2">
       <c r="A29" t="s">
         <v>39</v>
       </c>
@@ -969,7 +1596,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2">
       <c r="A30" t="s">
         <v>41</v>
       </c>
@@ -977,7 +1604,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -985,7 +1612,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2">
       <c r="A32" t="s">
         <v>45</v>
       </c>
@@ -993,7 +1620,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2">
       <c r="A33" t="s">
         <v>47</v>
       </c>
@@ -1001,7 +1628,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2">
       <c r="A34" t="s">
         <v>49</v>
       </c>
@@ -1009,7 +1636,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2">
       <c r="A35" t="s">
         <v>51</v>
       </c>
@@ -1017,7 +1644,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2">
       <c r="A36" t="s">
         <v>53</v>
       </c>
@@ -1025,7 +1652,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2">
       <c r="A37" t="s">
         <v>55</v>
       </c>
@@ -1033,7 +1660,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2">
       <c r="A38" t="s">
         <v>57</v>
       </c>
@@ -1041,7 +1668,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2">
       <c r="A39" t="s">
         <v>59</v>
       </c>
@@ -1049,7 +1676,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2">
       <c r="A40" t="s">
         <v>61</v>
       </c>
@@ -1057,7 +1684,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2">
       <c r="A41" t="s">
         <v>63</v>
       </c>
@@ -1065,7 +1692,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2">
       <c r="A42" t="s">
         <v>65</v>
       </c>
@@ -1073,7 +1700,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2">
       <c r="A43" t="s">
         <v>67</v>
       </c>
@@ -1081,7 +1708,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2">
       <c r="A44" t="s">
         <v>69</v>
       </c>
@@ -1089,7 +1716,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2">
       <c r="A45" t="s">
         <v>71</v>
       </c>
@@ -1097,7 +1724,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2">
       <c r="A46" t="s">
         <v>73</v>
       </c>
@@ -1105,7 +1732,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2">
       <c r="A47" t="s">
         <v>75</v>
       </c>
@@ -1113,12 +1740,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1">
       <c r="A48" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2">
       <c r="A49" t="s">
         <v>77</v>
       </c>
@@ -1126,7 +1753,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2">
       <c r="A50" t="s">
         <v>79</v>
       </c>
@@ -1134,17 +1761,17 @@
         <v>80</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1">
       <c r="A51" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1">
       <c r="A52" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2">
       <c r="A53" t="s">
         <v>83</v>
       </c>
@@ -1152,7 +1779,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2">
       <c r="A54" t="s">
         <v>85</v>
       </c>
@@ -1160,17 +1787,17 @@
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1">
       <c r="A55" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1">
       <c r="A56" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2">
       <c r="A57" t="s">
         <v>89</v>
       </c>
@@ -1178,7 +1805,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2">
       <c r="A58" t="s">
         <v>7</v>
       </c>
@@ -1186,42 +1813,42 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1">
       <c r="A59" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1">
       <c r="A60" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1">
       <c r="A61" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1">
       <c r="A62" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1">
       <c r="A63" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1">
       <c r="A64" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1">
       <c r="A65" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2">
       <c r="A66" t="s">
         <v>98</v>
       </c>
@@ -1229,17 +1856,17 @@
         <v>99</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:1">
       <c r="A67" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:1">
       <c r="A68" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2">
       <c r="A69" t="s">
         <v>102</v>
       </c>
@@ -1247,17 +1874,17 @@
         <v>99</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:1">
       <c r="A70" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:1">
       <c r="A71" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2">
       <c r="A72" t="s">
         <v>105</v>
       </c>
@@ -1265,17 +1892,17 @@
         <v>99</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:1">
       <c r="A73" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:1">
       <c r="A74" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2">
       <c r="A75" t="s">
         <v>108</v>
       </c>
@@ -1283,17 +1910,17 @@
         <v>99</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:1">
       <c r="A76" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:1">
       <c r="A77" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2">
       <c r="A78" t="s">
         <v>111</v>
       </c>
@@ -1301,7 +1928,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2">
       <c r="A79" t="s">
         <v>112</v>
       </c>
@@ -1309,12 +1936,12 @@
         <v>99</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:1">
       <c r="A80" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2">
       <c r="A81" t="s">
         <v>114</v>
       </c>
@@ -1322,7 +1949,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2">
       <c r="A82" t="s">
         <v>115</v>
       </c>
@@ -1330,7 +1957,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2">
       <c r="A83" t="s">
         <v>116</v>
       </c>
@@ -1338,7 +1965,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:2">
       <c r="A84" t="s">
         <v>118</v>
       </c>
@@ -1346,32 +1973,32 @@
         <v>119</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:1">
       <c r="A85" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:1">
       <c r="A86" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:1">
       <c r="A87" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:1">
       <c r="A88" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:1">
       <c r="A89" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2">
       <c r="A90" t="s">
         <v>125</v>
       </c>
@@ -1379,7 +2006,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2">
       <c r="A91" t="s">
         <v>127</v>
       </c>
@@ -1387,7 +2014,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:2">
       <c r="A92" t="s">
         <v>128</v>
       </c>
@@ -1395,7 +2022,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2">
       <c r="A93" t="s">
         <v>129</v>
       </c>
@@ -1403,7 +2030,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:1">
       <c r="A94" t="s">
         <v>130</v>
       </c>
@@ -1413,5 +2040,6 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>